<commit_message>
Improved CustomersView and fix views register x update, to fix payment
</commit_message>
<xml_diff>
--- a/api/public/xlsx/ativos/clientes_ativos.xlsx
+++ b/api/public/xlsx/ativos/clientes_ativos.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="10">
   <si>
     <t>Cliente</t>
   </si>
@@ -32,7 +32,7 @@
     <t>Status</t>
   </si>
   <si>
-    <t>Teste 1</t>
+    <t>Teste 1 alterado</t>
   </si>
   <si>
     <t>teste1@teste.com</t>
@@ -41,25 +41,10 @@
     <t>Ativo</t>
   </si>
   <si>
-    <t>Teste 2</t>
+    <t>Teste 1 alterado 2</t>
   </si>
   <si>
     <t>teste2@teste.com</t>
-  </si>
-  <si>
-    <t>Gabriel Kochem Ichazo</t>
-  </si>
-  <si>
-    <t>08805166901</t>
-  </si>
-  <si>
-    <t>gabikochem55@gmail.com</t>
-  </si>
-  <si>
-    <t>Laura Refosco</t>
-  </si>
-  <si>
-    <t>gabikochem15@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -399,7 +384,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -444,34 +429,6 @@
         <v>9</v>
       </c>
       <c r="E3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
-      <c r="A4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E4" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5">
-      <c r="A5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B5">
-        <v>11111111111111</v>
-      </c>
-      <c r="D5" t="s">
-        <v>14</v>
-      </c>
-      <c r="E5" t="s">
         <v>7</v>
       </c>
     </row>

</xml_diff>

<commit_message>
IMPROVED customers and products view, to make report products and to fix paymentform
</commit_message>
<xml_diff>
--- a/api/public/xlsx/ativos/clientes_ativos.xlsx
+++ b/api/public/xlsx/ativos/clientes_ativos.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="16">
   <si>
     <t>Cliente</t>
   </si>
@@ -41,10 +41,28 @@
     <t>Ativo</t>
   </si>
   <si>
-    <t>Teste 1 alterado 2</t>
+    <t>Teste 1</t>
   </si>
   <si>
     <t>teste2@teste.com</t>
+  </si>
+  <si>
+    <t>Teste</t>
+  </si>
+  <si>
+    <t>ga@a</t>
+  </si>
+  <si>
+    <t>teste grid</t>
+  </si>
+  <si>
+    <t>dgfg#@aa</t>
+  </si>
+  <si>
+    <t>teste cpf e cnpj</t>
+  </si>
+  <si>
+    <t>aaaaaaaaa@a</t>
   </si>
 </sst>
 </file>
@@ -384,7 +402,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -429,6 +447,51 @@
         <v>9</v>
       </c>
       <c r="E3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4">
+        <v>60880519111</v>
+      </c>
+      <c r="D4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5">
+        <v>42442424024</v>
+      </c>
+      <c r="D5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6">
+        <v>11111111111111</v>
+      </c>
+      <c r="C6">
+        <v>11111111111</v>
+      </c>
+      <c r="D6" t="s">
+        <v>15</v>
+      </c>
+      <c r="E6" t="s">
         <v>7</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Improved customers and products view, to fix payment
</commit_message>
<xml_diff>
--- a/api/public/xlsx/ativos/clientes_ativos.xlsx
+++ b/api/public/xlsx/ativos/clientes_ativos.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="15">
   <si>
     <t>Cliente</t>
   </si>
@@ -32,7 +32,7 @@
     <t>Status</t>
   </si>
   <si>
-    <t>Teste 1 alterado</t>
+    <t>Teste 1</t>
   </si>
   <si>
     <t>teste1@teste.com</t>
@@ -41,28 +41,25 @@
     <t>Ativo</t>
   </si>
   <si>
-    <t>Teste 1</t>
+    <t>Teste 2</t>
   </si>
   <si>
     <t>teste2@teste.com</t>
   </si>
   <si>
-    <t>Teste</t>
-  </si>
-  <si>
-    <t>ga@a</t>
-  </si>
-  <si>
-    <t>teste grid</t>
-  </si>
-  <si>
-    <t>dgfg#@aa</t>
-  </si>
-  <si>
-    <t>teste cpf e cnpj</t>
-  </si>
-  <si>
-    <t>aaaaaaaaa@a</t>
+    <t>kochem</t>
+  </si>
+  <si>
+    <t>Guinunespaludo246@gmail.com</t>
+  </si>
+  <si>
+    <t>TESTE 04</t>
+  </si>
+  <si>
+    <t>00000000000</t>
+  </si>
+  <si>
+    <t>teste@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -402,7 +399,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -454,8 +451,11 @@
       <c r="A4" t="s">
         <v>10</v>
       </c>
+      <c r="B4">
+        <v>13124124321234</v>
+      </c>
       <c r="C4">
-        <v>60880519111</v>
+        <v>11692388908</v>
       </c>
       <c r="D4" t="s">
         <v>11</v>
@@ -468,30 +468,13 @@
       <c r="A5" t="s">
         <v>12</v>
       </c>
-      <c r="C5">
-        <v>42442424024</v>
+      <c r="C5" t="s">
+        <v>13</v>
       </c>
       <c r="D5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5">
-      <c r="A6" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6">
-        <v>11111111111111</v>
-      </c>
-      <c r="C6">
-        <v>11111111111</v>
-      </c>
-      <c r="D6" t="s">
-        <v>15</v>
-      </c>
-      <c r="E6" t="s">
         <v>7</v>
       </c>
     </row>

</xml_diff>

<commit_message>
To fix products register and to fix payment service
</commit_message>
<xml_diff>
--- a/api/public/xlsx/ativos/clientes_ativos.xlsx
+++ b/api/public/xlsx/ativos/clientes_ativos.xlsx
@@ -32,7 +32,7 @@
     <t>Status</t>
   </si>
   <si>
-    <t>Teste 1</t>
+    <t>Teste 1aaaaaaaaaaaaaaaaaaaaaa</t>
   </si>
   <si>
     <t>teste1@teste.com</t>
@@ -47,19 +47,19 @@
     <t>teste2@teste.com</t>
   </si>
   <si>
-    <t>kochem</t>
-  </si>
-  <si>
-    <t>Guinunespaludo246@gmail.com</t>
-  </si>
-  <si>
-    <t>TESTE 04</t>
-  </si>
-  <si>
-    <t>00000000000</t>
-  </si>
-  <si>
-    <t>teste@gmail.com</t>
+    <t>Gabriel Kochem Ichazo</t>
+  </si>
+  <si>
+    <t>08805166901</t>
+  </si>
+  <si>
+    <t>gabikochem55@gmail.com</t>
+  </si>
+  <si>
+    <t>Laura Refosco</t>
+  </si>
+  <si>
+    <t>gabikochem15@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -451,14 +451,11 @@
       <c r="A4" t="s">
         <v>10</v>
       </c>
-      <c r="B4">
-        <v>13124124321234</v>
-      </c>
-      <c r="C4">
-        <v>11692388908</v>
+      <c r="C4" t="s">
+        <v>11</v>
       </c>
       <c r="D4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E4" t="s">
         <v>7</v>
@@ -466,10 +463,10 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" t="s">
         <v>13</v>
+      </c>
+      <c r="B5">
+        <v>11111111111111</v>
       </c>
       <c r="D5" t="s">
         <v>14</v>

</xml_diff>

<commit_message>
To improve: Finally payments forms PDV and others components
</commit_message>
<xml_diff>
--- a/api/public/xlsx/ativos/clientes_ativos.xlsx
+++ b/api/public/xlsx/ativos/clientes_ativos.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="7">
   <si>
     <t>Cliente</t>
   </si>
@@ -36,18 +36,6 @@
   </si>
   <si>
     <t>Ativo</t>
-  </si>
-  <si>
-    <t>Sgbr Sistemas</t>
-  </si>
-  <si>
-    <t>Inativo</t>
-  </si>
-  <si>
-    <t>teste</t>
-  </si>
-  <si>
-    <t>Teste2 aaaa</t>
   </si>
 </sst>
 </file>
@@ -387,7 +375,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -415,39 +403,6 @@
         <v>5</v>
       </c>
       <c r="D2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
-      <c r="A3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3">
-        <v>17089484000190</v>
-      </c>
-      <c r="D3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4">
-        <v>41390805000176</v>
-      </c>
-      <c r="D4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
-      <c r="A5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5">
-        <v>49478610000194</v>
-      </c>
-      <c r="D5" t="s">
         <v>6</v>
       </c>
     </row>

</xml_diff>

<commit_message>
To implement get color
</commit_message>
<xml_diff>
--- a/api/public/xlsx/ativos/clientes_ativos.xlsx
+++ b/api/public/xlsx/ativos/clientes_ativos.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="11">
   <si>
     <t>Cliente</t>
   </si>
@@ -36,6 +36,18 @@
   </si>
   <si>
     <t>Ativo</t>
+  </si>
+  <si>
+    <t>Sgbr Sistemas</t>
+  </si>
+  <si>
+    <t>Inativo</t>
+  </si>
+  <si>
+    <t>teste</t>
+  </si>
+  <si>
+    <t>Teste2 aaaa</t>
   </si>
 </sst>
 </file>
@@ -375,7 +387,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -403,6 +415,39 @@
         <v>5</v>
       </c>
       <c r="D2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3">
+        <v>17089484000190</v>
+      </c>
+      <c r="D3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4">
+        <v>41390805000176</v>
+      </c>
+      <c r="D4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5">
+        <v>49478610000194</v>
+      </c>
+      <c r="D5" t="s">
         <v>6</v>
       </c>
     </row>

</xml_diff>